<commit_message>
fix(documents): 판매계약서 금액 폰트 통일 — FOB 슬롯 전체(E23:G59) Arial
직전 수정은 E50:G59(합계+마지막 슬롯 3개)만 Arial 로 바꿔, 실제 채워지는
FOB 슬롯(first=23)은 Tahoma 로 남아 합계(Arial)와 폰트가 섞임 → 서버에서
FOB값과 합계 숫자의 우측정렬 위치가 달라 어긋나 보임(확대 확인). 슬롯 전
구간(23~52)+합계(53~59) E:G 를 Arial 로 통일. 서버 실물 Arial(mscorefonts)
과 맞물려 정확히 렌더. 3사 세트 적용.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/templates/heyman/sales_contract.xlsx
+++ b/resources/templates/heyman/sales_contract.xlsx
@@ -524,7 +524,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color rgb="FFAEABAB"/>
+      </left>
       <right/>
       <top style="thin">
         <color rgb="FFAEABAB"/>
@@ -535,9 +537,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFAEABAB"/>
-      </left>
+      <left/>
       <right/>
       <top style="thin">
         <color rgb="FFAEABAB"/>
@@ -628,19 +628,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFAEABAB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFAEABAB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -797,30 +784,8 @@
       <top style="thin">
         <color rgb="FFAEABAB"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFAEABAB"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFAEABAB"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFAEABAB"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
+      <bottom style="thin">
+        <color rgb="FFAEABAB"/>
       </bottom>
       <diagonal/>
     </border>
@@ -832,6 +797,41 @@
       <top style="thin">
         <color rgb="FFAEABAB"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAEABAB"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFAEABAB"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFAEABAB"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAEABAB"/>
+      </top>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
@@ -841,7 +841,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="100">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
@@ -861,9 +861,6 @@
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="6" numFmtId="165" fillId="3" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
-    </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
@@ -877,25 +874,25 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="7" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="8" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="9" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="8" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="9" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="10" numFmtId="0" fillId="4" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="11" numFmtId="0" fillId="5" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="11" numFmtId="0" fillId="5" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="12" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="12" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="12" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="5" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="14" fillId="0" borderId="5" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="0"/>
@@ -912,7 +909,6 @@
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="7" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
@@ -922,27 +918,27 @@
     <xf xfId="0" fontId="4" numFmtId="0" fillId="6" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="7" borderId="12" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="7" borderId="11" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="7" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="7" borderId="13" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="7" borderId="12" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="6" numFmtId="49" fillId="3" borderId="10" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
+    <xf xfId="0" fontId="6" numFmtId="49" fillId="3" borderId="13" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="49" fillId="3" borderId="2" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="6" numFmtId="49" fillId="3" borderId="14" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="6" numFmtId="49" fillId="3" borderId="2" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
-    </xf>
     <xf xfId="0" fontId="6" numFmtId="49" fillId="3" borderId="15" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="6" numFmtId="49" fillId="3" borderId="16" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="13" numFmtId="49" fillId="7" borderId="17" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="13" numFmtId="49" fillId="7" borderId="16" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="10" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
@@ -965,7 +961,7 @@
     <xf xfId="0" fontId="17" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="18" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
@@ -981,15 +977,18 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="16" numFmtId="14" fillId="0" borderId="5" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="16" numFmtId="0" fillId="0" borderId="18" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf xfId="0" fontId="16" numFmtId="0" fillId="0" borderId="17" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="18" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="12" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="19" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="13" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
-    </xf>
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="20" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
@@ -999,8 +998,8 @@
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="22" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="23" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="18" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="19" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
@@ -1008,13 +1007,10 @@
     <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="20" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="21" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="23" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="20" numFmtId="0" fillId="2" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="2" borderId="22" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="20" numFmtId="0" fillId="2" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="21" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
@@ -1024,16 +1020,16 @@
     <xf xfId="0" fontId="20" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
+    <xf xfId="0" fontId="22" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="22" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="22" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
     <xf xfId="0" fontId="22" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="22" numFmtId="14" fillId="0" borderId="4" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="22" numFmtId="14" fillId="0" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="23" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
@@ -1045,36 +1041,36 @@
     <xf xfId="0" fontId="6" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="22" numFmtId="14" fillId="0" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="8" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="9" numFmtId="0" fillId="0" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="22" numFmtId="14" fillId="0" borderId="4" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="8" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="9" numFmtId="0" fillId="0" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="5" borderId="24" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="5" borderId="23" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="14" numFmtId="0" fillId="8" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="165" fillId="3" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="1" numFmtId="165" fillId="3" borderId="4" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="11" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="165" fillId="7" borderId="19" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="24" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="165" fillId="7" borderId="18" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="165" fillId="7" borderId="13" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="1" numFmtId="165" fillId="7" borderId="12" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="7" borderId="25" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="165" fillId="0" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="1" numFmtId="165" fillId="0" borderId="4" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="165" fillId="0" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
     <xf xfId="0" fontId="1" numFmtId="165" fillId="7" borderId="26" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
@@ -1082,17 +1078,17 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="7" borderId="28" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="165" fillId="6" borderId="20" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
     <xf xfId="0" fontId="1" numFmtId="165" fillId="6" borderId="21" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="165" fillId="6" borderId="22" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="6" borderId="22" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="2" numFmtId="165" fillId="9" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="6" borderId="23" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
     <xf xfId="0" fontId="2" numFmtId="165" fillId="9" borderId="4" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="165" fillId="9" borderId="3" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="6" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
@@ -1392,19 +1388,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" customHeight="1" ht="53.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
       <c r="H1"/>
     </row>
     <row r="2" spans="1:8" customHeight="1" ht="21">
-      <c r="A2" s="47"/>
+      <c r="A2" s="45"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -1412,246 +1408,246 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" customHeight="1" ht="24">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="50"/>
-      <c r="C3" s="50"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="50"/>
-      <c r="F3" s="50"/>
-      <c r="G3" s="50"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
       <c r="H3"/>
     </row>
     <row r="4" spans="1:8" customHeight="1" ht="18">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50"/>
-      <c r="G4" s="50"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
       <c r="H4"/>
     </row>
     <row r="5" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A5" s="50" t="s">
+      <c r="A5" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
       <c r="H5"/>
     </row>
     <row r="6" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A6" s="49"/>
-      <c r="B6" s="49"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
+      <c r="A6" s="47"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
       <c r="H6"/>
     </row>
-    <row r="7" spans="1:8" customHeight="1" ht="18" s="48" customFormat="1">
-      <c r="A7" s="70" t="s">
+    <row r="7" spans="1:8" customHeight="1" ht="18" s="46" customFormat="1">
+      <c r="A7" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="71"/>
-      <c r="C7" s="72" t="s">
+      <c r="B7" s="69"/>
+      <c r="C7" s="70" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="73" t="s">
+      <c r="D7" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="74" t="s">
+      <c r="E7" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="75"/>
-      <c r="G7" s="71"/>
-      <c r="H7" s="48"/>
-    </row>
-    <row r="8" spans="1:8" customHeight="1" ht="18" s="48" customFormat="1">
-      <c r="A8" s="70" t="s">
+      <c r="F7" s="73"/>
+      <c r="G7" s="69"/>
+      <c r="H7" s="46"/>
+    </row>
+    <row r="8" spans="1:8" customHeight="1" ht="18" s="46" customFormat="1">
+      <c r="A8" s="68" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="71"/>
-      <c r="C8" s="78" t="s">
+      <c r="B8" s="69"/>
+      <c r="C8" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="73" t="s">
+      <c r="D8" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="74" t="s">
+      <c r="E8" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="75"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="48"/>
-    </row>
-    <row r="9" spans="1:8" customHeight="1" ht="18" s="48" customFormat="1">
-      <c r="A9" s="70" t="s">
+      <c r="F8" s="73"/>
+      <c r="G8" s="69"/>
+      <c r="H8" s="46"/>
+    </row>
+    <row r="9" spans="1:8" customHeight="1" ht="18" s="46" customFormat="1">
+      <c r="A9" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="71"/>
-      <c r="C9" s="74" t="s">
+      <c r="B9" s="69"/>
+      <c r="C9" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="75"/>
-      <c r="E9" s="75"/>
-      <c r="F9" s="75"/>
-      <c r="G9" s="76"/>
-      <c r="H9" s="48"/>
-    </row>
-    <row r="10" spans="1:8" customHeight="1" ht="18" s="48" customFormat="1">
-      <c r="A10" s="70" t="s">
+      <c r="D9" s="73"/>
+      <c r="E9" s="73"/>
+      <c r="F9" s="73"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="46"/>
+    </row>
+    <row r="10" spans="1:8" customHeight="1" ht="18" s="46" customFormat="1">
+      <c r="A10" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="71"/>
-      <c r="C10" s="74" t="s">
+      <c r="B10" s="69"/>
+      <c r="C10" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="75"/>
-      <c r="E10" s="75"/>
-      <c r="F10" s="75"/>
-      <c r="G10" s="76"/>
-      <c r="H10" s="48"/>
-    </row>
-    <row r="11" spans="1:8" customHeight="1" ht="18" s="48" customFormat="1">
-      <c r="A11" s="70" t="s">
+      <c r="D10" s="73"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="74"/>
+      <c r="H10" s="46"/>
+    </row>
+    <row r="11" spans="1:8" customHeight="1" ht="18" s="46" customFormat="1">
+      <c r="A11" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="71"/>
-      <c r="C11" s="74" t="s">
+      <c r="B11" s="69"/>
+      <c r="C11" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="75"/>
-      <c r="E11" s="75"/>
-      <c r="F11" s="75"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="48"/>
-    </row>
-    <row r="12" spans="1:8" customHeight="1" ht="18" s="48" customFormat="1">
-      <c r="A12" s="70" t="s">
+      <c r="D11" s="73"/>
+      <c r="E11" s="73"/>
+      <c r="F11" s="73"/>
+      <c r="G11" s="74"/>
+      <c r="H11" s="46"/>
+    </row>
+    <row r="12" spans="1:8" customHeight="1" ht="18" s="46" customFormat="1">
+      <c r="A12" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="71"/>
-      <c r="C12" s="72" t="s">
+      <c r="B12" s="69"/>
+      <c r="C12" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="73" t="s">
+      <c r="D12" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="77" t="str">
+      <c r="E12" s="75" t="str">
         <f>TODAY()</f>
         <v>0</v>
       </c>
-      <c r="F12" s="81"/>
-      <c r="G12" s="71"/>
-      <c r="H12" s="48"/>
+      <c r="F12" s="79"/>
+      <c r="G12" s="69"/>
+      <c r="H12" s="46"/>
     </row>
     <row r="13" spans="1:8" customHeight="1" ht="15">
-      <c r="A13" s="46"/>
+      <c r="A13" s="44"/>
       <c r="H13"/>
     </row>
     <row r="14" spans="1:8" customHeight="1" ht="15">
-      <c r="A14" s="45"/>
+      <c r="A14" s="43"/>
       <c r="C14" s="2"/>
       <c r="D14" s="3"/>
       <c r="H14"/>
     </row>
     <row r="15" spans="1:8" customHeight="1" ht="17.25">
-      <c r="A15" s="20" t="s">
+      <c r="A15" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="22"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="21"/>
       <c r="H15"/>
     </row>
     <row r="16" spans="1:8" customHeight="1" ht="17.25">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="14"/>
+      <c r="B16" s="13"/>
       <c r="C16" s="4" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="51"/>
-      <c r="G16" s="14"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="13"/>
       <c r="H16"/>
     </row>
     <row r="17" spans="1:8" customHeight="1" ht="17.25">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="14"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="82"/>
-      <c r="G17" s="14"/>
+      <c r="F17" s="80"/>
+      <c r="G17" s="13"/>
       <c r="H17"/>
     </row>
     <row r="18" spans="1:8" customHeight="1" ht="17.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="14"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="4" t="s">
         <v>31</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="F18" s="83"/>
-      <c r="G18" s="14"/>
+      <c r="F18" s="81"/>
+      <c r="G18" s="13"/>
       <c r="H18"/>
     </row>
     <row r="19" spans="1:8" customHeight="1" ht="17.25">
-      <c r="A19" s="66" t="s">
+      <c r="A19" s="64" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="67"/>
-      <c r="C19" s="60" t="s">
+      <c r="B19" s="65"/>
+      <c r="C19" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="61"/>
-      <c r="E19" s="61"/>
-      <c r="F19" s="61"/>
-      <c r="G19" s="62"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="59"/>
+      <c r="G19" s="60"/>
       <c r="H19"/>
     </row>
     <row r="20" spans="1:8" customHeight="1" ht="17.25">
-      <c r="A20" s="68"/>
-      <c r="B20" s="69"/>
-      <c r="C20" s="63"/>
-      <c r="D20" s="64"/>
-      <c r="E20" s="64"/>
-      <c r="F20" s="64"/>
-      <c r="G20" s="65"/>
+      <c r="A20" s="66"/>
+      <c r="B20" s="67"/>
+      <c r="C20" s="61"/>
+      <c r="D20" s="62"/>
+      <c r="E20" s="62"/>
+      <c r="F20" s="62"/>
+      <c r="G20" s="63"/>
       <c r="H20"/>
     </row>
     <row r="21" spans="1:8" customHeight="1" ht="12.75">
@@ -1661,409 +1657,409 @@
       <c r="H21"/>
     </row>
     <row r="22" spans="1:8" customHeight="1" ht="23.25">
-      <c r="A22" s="25" t="s">
+      <c r="A22" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="B22" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="C22" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="26" t="s">
+      <c r="D22" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="27" t="s">
+      <c r="E22" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="F22" s="84"/>
-      <c r="G22" s="28"/>
+      <c r="F22" s="82"/>
+      <c r="G22" s="27"/>
       <c r="H22"/>
     </row>
     <row r="23" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A23" s="29"/>
+      <c r="A23" s="28"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="10"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="84"/>
+      <c r="F23" s="84"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="9"/>
     </row>
     <row r="24" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A24" s="29"/>
+      <c r="A24" s="28"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="84"/>
+      <c r="F24" s="84"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="9"/>
     </row>
     <row r="25" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A25" s="29"/>
+      <c r="A25" s="28"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="10"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="84"/>
+      <c r="F25" s="84"/>
+      <c r="G25" s="85"/>
+      <c r="H25" s="9"/>
     </row>
     <row r="26" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A26" s="29"/>
+      <c r="A26" s="28"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="84"/>
+      <c r="F26" s="84"/>
+      <c r="G26" s="85"/>
+      <c r="H26" s="10"/>
     </row>
     <row r="27" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A27" s="29"/>
+      <c r="A27" s="28"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="84"/>
+      <c r="F27" s="84"/>
+      <c r="G27" s="85"/>
+      <c r="H27" s="10"/>
     </row>
     <row r="28" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A28" s="29"/>
+      <c r="A28" s="28"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="84"/>
+      <c r="F28" s="84"/>
+      <c r="G28" s="85"/>
+      <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A29" s="29"/>
+      <c r="A29" s="28"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="30"/>
-      <c r="H29" s="10"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="84"/>
+      <c r="F29" s="84"/>
+      <c r="G29" s="85"/>
+      <c r="H29" s="9"/>
     </row>
     <row r="30" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A30" s="29"/>
+      <c r="A30" s="28"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="30"/>
-      <c r="H30" s="10"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="84"/>
+      <c r="F30" s="84"/>
+      <c r="G30" s="85"/>
+      <c r="H30" s="9"/>
     </row>
     <row r="31" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A31" s="29"/>
+      <c r="A31" s="28"/>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="30"/>
-      <c r="H31" s="10"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="84"/>
+      <c r="F31" s="84"/>
+      <c r="G31" s="85"/>
+      <c r="H31" s="9"/>
     </row>
     <row r="32" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A32" s="29"/>
+      <c r="A32" s="28"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="10"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="84"/>
+      <c r="F32" s="84"/>
+      <c r="G32" s="85"/>
+      <c r="H32" s="9"/>
     </row>
     <row r="33" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A33" s="29"/>
+      <c r="A33" s="28"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="10"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="84"/>
+      <c r="F33" s="84"/>
+      <c r="G33" s="85"/>
+      <c r="H33" s="9"/>
     </row>
     <row r="34" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A34" s="29"/>
+      <c r="A34" s="28"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="10"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="84"/>
+      <c r="F34" s="84"/>
+      <c r="G34" s="85"/>
+      <c r="H34" s="9"/>
     </row>
     <row r="35" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A35" s="29"/>
+      <c r="A35" s="28"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="30"/>
-      <c r="H35" s="10"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="84"/>
+      <c r="F35" s="84"/>
+      <c r="G35" s="85"/>
+      <c r="H35" s="9"/>
     </row>
     <row r="36" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A36" s="29"/>
+      <c r="A36" s="28"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="30"/>
-      <c r="H36" s="10"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="84"/>
+      <c r="F36" s="84"/>
+      <c r="G36" s="85"/>
+      <c r="H36" s="9"/>
     </row>
     <row r="37" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A37" s="29"/>
+      <c r="A37" s="28"/>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="30"/>
-      <c r="H37" s="10"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="84"/>
+      <c r="F37" s="84"/>
+      <c r="G37" s="85"/>
+      <c r="H37" s="9"/>
     </row>
     <row r="38" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A38" s="29"/>
+      <c r="A38" s="28"/>
       <c r="B38" s="8"/>
       <c r="C38" s="8"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="30"/>
-      <c r="H38" s="10"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="84"/>
+      <c r="F38" s="84"/>
+      <c r="G38" s="85"/>
+      <c r="H38" s="9"/>
     </row>
     <row r="39" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A39" s="29"/>
+      <c r="A39" s="28"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="30"/>
-      <c r="H39" s="10"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="84"/>
+      <c r="F39" s="84"/>
+      <c r="G39" s="85"/>
+      <c r="H39" s="9"/>
     </row>
     <row r="40" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A40" s="29"/>
+      <c r="A40" s="28"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="10"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="84"/>
+      <c r="F40" s="84"/>
+      <c r="G40" s="85"/>
+      <c r="H40" s="9"/>
     </row>
     <row r="41" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A41" s="29"/>
+      <c r="A41" s="28"/>
       <c r="B41" s="8"/>
       <c r="C41" s="8"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="30"/>
-      <c r="H41" s="10"/>
+      <c r="D41" s="11"/>
+      <c r="E41" s="84"/>
+      <c r="F41" s="84"/>
+      <c r="G41" s="85"/>
+      <c r="H41" s="9"/>
     </row>
     <row r="42" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A42" s="29"/>
+      <c r="A42" s="28"/>
       <c r="B42" s="8"/>
       <c r="C42" s="8"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="9"/>
-      <c r="F42" s="9"/>
-      <c r="G42" s="30"/>
-      <c r="H42" s="10"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="84"/>
+      <c r="F42" s="84"/>
+      <c r="G42" s="85"/>
+      <c r="H42" s="9"/>
     </row>
     <row r="43" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A43" s="29"/>
+      <c r="A43" s="28"/>
       <c r="B43" s="8"/>
       <c r="C43" s="8"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="30"/>
-      <c r="H43" s="10"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="84"/>
+      <c r="F43" s="84"/>
+      <c r="G43" s="85"/>
+      <c r="H43" s="9"/>
     </row>
     <row r="44" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A44" s="29"/>
+      <c r="A44" s="28"/>
       <c r="B44" s="8"/>
       <c r="C44" s="8"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="30"/>
-      <c r="H44" s="10"/>
+      <c r="D44" s="11"/>
+      <c r="E44" s="84"/>
+      <c r="F44" s="84"/>
+      <c r="G44" s="85"/>
+      <c r="H44" s="9"/>
     </row>
     <row r="45" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A45" s="29"/>
+      <c r="A45" s="28"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="30"/>
-      <c r="H45" s="10"/>
+      <c r="D45" s="11"/>
+      <c r="E45" s="84"/>
+      <c r="F45" s="84"/>
+      <c r="G45" s="85"/>
+      <c r="H45" s="9"/>
     </row>
     <row r="46" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A46" s="29"/>
+      <c r="A46" s="28"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="30"/>
-      <c r="H46" s="10"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="84"/>
+      <c r="F46" s="84"/>
+      <c r="G46" s="85"/>
+      <c r="H46" s="9"/>
     </row>
     <row r="47" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A47" s="29"/>
+      <c r="A47" s="28"/>
       <c r="B47" s="8"/>
       <c r="C47" s="8"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="30"/>
-      <c r="H47" s="10"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="84"/>
+      <c r="F47" s="84"/>
+      <c r="G47" s="85"/>
+      <c r="H47" s="9"/>
     </row>
     <row r="48" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A48" s="29"/>
+      <c r="A48" s="28"/>
       <c r="B48" s="8"/>
       <c r="C48" s="8"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="30"/>
-      <c r="H48" s="10"/>
+      <c r="D48" s="11"/>
+      <c r="E48" s="84"/>
+      <c r="F48" s="84"/>
+      <c r="G48" s="85"/>
+      <c r="H48" s="9"/>
     </row>
     <row r="49" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A49" s="29"/>
+      <c r="A49" s="28"/>
       <c r="B49" s="8"/>
       <c r="C49" s="8"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="30"/>
-      <c r="H49" s="10"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="84"/>
+      <c r="F49" s="84"/>
+      <c r="G49" s="85"/>
+      <c r="H49" s="9"/>
     </row>
     <row r="50" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A50" s="29"/>
+      <c r="A50" s="28"/>
       <c r="B50" s="8"/>
       <c r="C50" s="8"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="86"/>
-      <c r="F50" s="86"/>
-      <c r="G50" s="87"/>
-      <c r="H50" s="10"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="84"/>
+      <c r="F50" s="84"/>
+      <c r="G50" s="85"/>
+      <c r="H50" s="9"/>
     </row>
     <row r="51" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A51" s="29"/>
+      <c r="A51" s="28"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="86"/>
-      <c r="F51" s="86"/>
-      <c r="G51" s="87"/>
-      <c r="H51" s="10"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="84"/>
+      <c r="F51" s="84"/>
+      <c r="G51" s="85"/>
+      <c r="H51" s="9"/>
     </row>
     <row r="52" spans="1:8" customHeight="1" ht="15.75">
-      <c r="A52" s="29"/>
+      <c r="A52" s="28"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="86"/>
-      <c r="F52" s="86"/>
-      <c r="G52" s="87"/>
-      <c r="H52" s="10"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="84"/>
+      <c r="F52" s="84"/>
+      <c r="G52" s="85"/>
+      <c r="H52" s="9"/>
     </row>
     <row r="53" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A53" s="34"/>
-      <c r="B53" s="35"/>
-      <c r="C53" s="35"/>
-      <c r="D53" s="36" t="s">
+      <c r="A53" s="32"/>
+      <c r="B53" s="33"/>
+      <c r="C53" s="33"/>
+      <c r="D53" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="E53" s="88"/>
-      <c r="F53" s="89"/>
-      <c r="G53" s="90"/>
+      <c r="E53" s="86"/>
+      <c r="F53" s="87"/>
+      <c r="G53" s="88"/>
       <c r="H53"/>
     </row>
     <row r="54" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A54" s="37"/>
-      <c r="B54" s="40"/>
-      <c r="C54" s="40"/>
-      <c r="D54" s="13" t="s">
+      <c r="A54" s="35"/>
+      <c r="B54" s="38"/>
+      <c r="C54" s="38"/>
+      <c r="D54" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="E54" s="91"/>
-      <c r="F54" s="92"/>
-      <c r="G54" s="87"/>
+      <c r="E54" s="89"/>
+      <c r="F54" s="90"/>
+      <c r="G54" s="85"/>
       <c r="H54"/>
     </row>
     <row r="55" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A55" s="43"/>
-      <c r="B55" s="79" t="s">
+      <c r="A55" s="41"/>
+      <c r="B55" s="77" t="s">
         <v>43</v>
       </c>
-      <c r="C55" s="79"/>
-      <c r="D55" s="39" t="s">
+      <c r="C55" s="77"/>
+      <c r="D55" s="37" t="s">
         <v>44</v>
       </c>
-      <c r="E55" s="91"/>
-      <c r="F55" s="92"/>
-      <c r="G55" s="87"/>
+      <c r="E55" s="89"/>
+      <c r="F55" s="90"/>
+      <c r="G55" s="85"/>
       <c r="H55"/>
     </row>
     <row r="56" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A56" s="31"/>
-      <c r="B56" s="80" t="s">
+      <c r="A56" s="29"/>
+      <c r="B56" s="78" t="s">
         <v>45</v>
       </c>
-      <c r="C56" s="80"/>
-      <c r="D56" s="39"/>
-      <c r="E56" s="91"/>
-      <c r="F56" s="92"/>
-      <c r="G56" s="87"/>
+      <c r="C56" s="78"/>
+      <c r="D56" s="37"/>
+      <c r="E56" s="89"/>
+      <c r="F56" s="90"/>
+      <c r="G56" s="85"/>
       <c r="H56"/>
     </row>
     <row r="57" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A57" s="38"/>
-      <c r="B57" s="41"/>
-      <c r="C57" s="41"/>
-      <c r="D57" s="42" t="s">
+      <c r="A57" s="36"/>
+      <c r="B57" s="39"/>
+      <c r="C57" s="39"/>
+      <c r="D57" s="40" t="s">
         <v>46</v>
       </c>
-      <c r="E57" s="93"/>
-      <c r="F57" s="94"/>
-      <c r="G57" s="95"/>
+      <c r="E57" s="91"/>
+      <c r="F57" s="92"/>
+      <c r="G57" s="93"/>
       <c r="H57"/>
     </row>
     <row r="58" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A58" s="55"/>
-      <c r="B58" s="56"/>
-      <c r="C58" s="55"/>
-      <c r="D58" s="33" t="s">
+      <c r="A58" s="53"/>
+      <c r="B58" s="54"/>
+      <c r="C58" s="53"/>
+      <c r="D58" s="31" t="s">
         <v>47</v>
       </c>
-      <c r="E58" s="96"/>
-      <c r="F58" s="97"/>
-      <c r="G58" s="98"/>
+      <c r="E58" s="94"/>
+      <c r="F58" s="95"/>
+      <c r="G58" s="96"/>
       <c r="H58"/>
     </row>
     <row r="59" spans="1:8" customHeight="1" ht="18.75">
-      <c r="A59" s="55"/>
-      <c r="B59" s="55"/>
-      <c r="C59" s="55"/>
-      <c r="D59" s="32" t="s">
+      <c r="A59" s="53"/>
+      <c r="B59" s="53"/>
+      <c r="C59" s="53"/>
+      <c r="D59" s="30" t="s">
         <v>48</v>
       </c>
-      <c r="E59" s="99"/>
-      <c r="F59" s="100"/>
-      <c r="G59" s="101"/>
+      <c r="E59" s="97"/>
+      <c r="F59" s="98"/>
+      <c r="G59" s="99"/>
       <c r="H59"/>
     </row>
     <row r="60" spans="1:8" customHeight="1" ht="12.75">
@@ -2076,75 +2072,75 @@
       <c r="H62"/>
     </row>
     <row r="63" spans="1:8" customHeight="1" ht="24">
-      <c r="B63" s="44" t="s">
+      <c r="B63" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="C63" s="44"/>
-      <c r="E63" s="85" t="s">
+      <c r="C63" s="42"/>
+      <c r="E63" s="83" t="s">
         <v>50</v>
       </c>
-      <c r="F63" s="85"/>
+      <c r="F63" s="83"/>
       <c r="H63"/>
     </row>
     <row r="64" spans="1:8" customHeight="1" ht="12.75">
-      <c r="B64" s="23"/>
-      <c r="C64" s="24"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
+      <c r="B64" s="22"/>
+      <c r="C64" s="23"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
       <c r="H64"/>
     </row>
     <row r="65" spans="1:8" customHeight="1" ht="12.75">
       <c r="H65"/>
     </row>
     <row r="66" spans="1:8" customHeight="1" ht="12.75">
-      <c r="B66" s="53" t="s">
+      <c r="B66" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="C66" s="53"/>
-      <c r="E66" s="53" t="s">
+      <c r="C66" s="51"/>
+      <c r="E66" s="51" t="s">
         <v>52</v>
       </c>
-      <c r="F66" s="53"/>
+      <c r="F66" s="51"/>
       <c r="H66"/>
     </row>
     <row r="67" spans="1:8" customHeight="1" ht="12.75">
-      <c r="B67" s="54"/>
-      <c r="C67" s="54"/>
-      <c r="E67" s="54"/>
-      <c r="F67" s="54"/>
+      <c r="B67" s="52"/>
+      <c r="C67" s="52"/>
+      <c r="E67" s="52"/>
+      <c r="F67" s="52"/>
       <c r="H67"/>
     </row>
     <row r="68" spans="1:8" customHeight="1" ht="20.25">
-      <c r="B68" s="59" t="s">
+      <c r="B68" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="C68" s="59"/>
-      <c r="E68" s="59" t="s">
+      <c r="C68" s="57"/>
+      <c r="E68" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="F68" s="59"/>
+      <c r="F68" s="57"/>
       <c r="H68"/>
     </row>
     <row r="69" spans="1:8" customHeight="1" ht="20.25">
-      <c r="B69" s="57" t="s">
+      <c r="B69" s="55" t="s">
         <v>55</v>
       </c>
-      <c r="C69" s="58"/>
-      <c r="E69" s="59" t="s">
+      <c r="C69" s="56"/>
+      <c r="E69" s="57" t="s">
         <v>56</v>
       </c>
-      <c r="F69" s="59"/>
+      <c r="F69" s="57"/>
       <c r="H69"/>
     </row>
     <row r="70" spans="1:8" customHeight="1" ht="20.25">
-      <c r="B70" s="57" t="s">
+      <c r="B70" s="55" t="s">
         <v>57</v>
       </c>
-      <c r="C70" s="58"/>
-      <c r="E70" s="59" t="s">
+      <c r="C70" s="56"/>
+      <c r="E70" s="57" t="s">
         <v>58</v>
       </c>
-      <c r="F70" s="59"/>
+      <c r="F70" s="57"/>
       <c r="H70"/>
     </row>
     <row r="71" spans="1:8" customHeight="1" ht="12.75">
@@ -2157,15 +2153,15 @@
     </row>
     <row r="72" spans="1:8" customHeight="1" ht="12.75">
       <c r="A72"/>
-      <c r="B72" s="52" t="s">
+      <c r="B72" s="50" t="s">
         <v>59</v>
       </c>
       <c r="C72"/>
       <c r="D72"/>
-      <c r="E72" s="52" t="s">
+      <c r="E72" s="50" t="s">
         <v>59</v>
       </c>
-      <c r="F72" s="52"/>
+      <c r="F72" s="50"/>
       <c r="H72"/>
     </row>
     <row r="73" spans="1:8">

</xml_diff>